<commit_message>
Update exam ticket journal
</commit_message>
<xml_diff>
--- a/journal.xlsx
+++ b/journal.xlsx
@@ -53,6 +53,12 @@
   </x:si>
   <x:si>
     <x:t>Алексеев</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Елизавета</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Гырдымова</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -430,7 +436,7 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="13.853482" style="0" customWidth="1"/>
-    <x:col min="2" max="2" width="10.282054" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="11.853482" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="14.139196" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="18.567768" style="0" customWidth="1"/>
   </x:cols>
@@ -517,6 +523,20 @@
       </x:c>
       <x:c r="D6" s="2">
         <x:v>46274.5133485185</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:4">
+      <x:c r="A7" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B7" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="C7" s="0">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D7" s="2">
+        <x:v>46287.6702784722</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>